<commit_message>
hotfix data set RDPatentValid
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/tech-yearbook/part08-output/01-patent/03-valid/2010.xlsx
+++ b/data-raw/data-tidy/tech-yearbook/part08-output/01-patent/03-valid/2010.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">variables</t>
   </si>
   <si>
-    <t xml:space="preserve">全   国</t>
+    <t xml:space="preserve">全国</t>
   </si>
   <si>
     <t xml:space="preserve">2010</t>
@@ -44,118 +44,118 @@
     <t xml:space="preserve">件</t>
   </si>
   <si>
-    <t xml:space="preserve">v4_cg_zlsq2_hj</t>
+    <t xml:space="preserve">v4_cg_zlsyx_hj</t>
   </si>
   <si>
     <t xml:space="preserve">发明</t>
   </si>
   <si>
-    <t xml:space="preserve">v4_cg_zlsq2_fm</t>
+    <t xml:space="preserve">v4_cg_zlsyx_fm</t>
   </si>
   <si>
     <t xml:space="preserve">实用新型</t>
   </si>
   <si>
-    <t xml:space="preserve">v4_cg_zlsq2_syxx</t>
+    <t xml:space="preserve">v4_cg_zlsyx_syxx</t>
   </si>
   <si>
     <t xml:space="preserve">外观设计</t>
   </si>
   <si>
-    <t xml:space="preserve">v4_cg_zlsq2_wgsj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">北   京</t>
-  </si>
-  <si>
-    <t xml:space="preserve">天   津</t>
-  </si>
-  <si>
-    <t xml:space="preserve">河   北</t>
-  </si>
-  <si>
-    <t xml:space="preserve">山   西</t>
-  </si>
-  <si>
-    <t xml:space="preserve">内蒙 古</t>
-  </si>
-  <si>
-    <t xml:space="preserve">辽   宁</t>
-  </si>
-  <si>
-    <t xml:space="preserve">吉   林</t>
-  </si>
-  <si>
-    <t xml:space="preserve">黑龙 江</t>
-  </si>
-  <si>
-    <t xml:space="preserve">上   海</t>
-  </si>
-  <si>
-    <t xml:space="preserve">江   苏</t>
-  </si>
-  <si>
-    <t xml:space="preserve">浙   江</t>
-  </si>
-  <si>
-    <t xml:space="preserve">安   徽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">福   建</t>
-  </si>
-  <si>
-    <t xml:space="preserve">江   西</t>
-  </si>
-  <si>
-    <t xml:space="preserve">山   东</t>
-  </si>
-  <si>
-    <t xml:space="preserve">河   南</t>
-  </si>
-  <si>
-    <t xml:space="preserve">湖   北</t>
-  </si>
-  <si>
-    <t xml:space="preserve">湖   南</t>
-  </si>
-  <si>
-    <t xml:space="preserve">广   东</t>
-  </si>
-  <si>
-    <t xml:space="preserve">广   西</t>
-  </si>
-  <si>
-    <t xml:space="preserve">海   南</t>
-  </si>
-  <si>
-    <t xml:space="preserve">重   庆</t>
-  </si>
-  <si>
-    <t xml:space="preserve">四   川</t>
-  </si>
-  <si>
-    <t xml:space="preserve">贵   州</t>
-  </si>
-  <si>
-    <t xml:space="preserve">云   南</t>
-  </si>
-  <si>
-    <t xml:space="preserve">西   藏</t>
-  </si>
-  <si>
-    <t xml:space="preserve">陕   西</t>
-  </si>
-  <si>
-    <t xml:space="preserve">甘   肃</t>
-  </si>
-  <si>
-    <t xml:space="preserve">青   海</t>
-  </si>
-  <si>
-    <t xml:space="preserve">宁   夏</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新   疆</t>
+    <t xml:space="preserve">v4_cg_zlsyx_wgsj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">北京</t>
+  </si>
+  <si>
+    <t xml:space="preserve">天津</t>
+  </si>
+  <si>
+    <t xml:space="preserve">河北</t>
+  </si>
+  <si>
+    <t xml:space="preserve">山西</t>
+  </si>
+  <si>
+    <t xml:space="preserve">内蒙古</t>
+  </si>
+  <si>
+    <t xml:space="preserve">辽宁</t>
+  </si>
+  <si>
+    <t xml:space="preserve">吉林</t>
+  </si>
+  <si>
+    <t xml:space="preserve">黑龙江</t>
+  </si>
+  <si>
+    <t xml:space="preserve">上海</t>
+  </si>
+  <si>
+    <t xml:space="preserve">江苏</t>
+  </si>
+  <si>
+    <t xml:space="preserve">浙江</t>
+  </si>
+  <si>
+    <t xml:space="preserve">安徽</t>
+  </si>
+  <si>
+    <t xml:space="preserve">福建</t>
+  </si>
+  <si>
+    <t xml:space="preserve">江西</t>
+  </si>
+  <si>
+    <t xml:space="preserve">山东</t>
+  </si>
+  <si>
+    <t xml:space="preserve">河南</t>
+  </si>
+  <si>
+    <t xml:space="preserve">湖北</t>
+  </si>
+  <si>
+    <t xml:space="preserve">湖南</t>
+  </si>
+  <si>
+    <t xml:space="preserve">广东</t>
+  </si>
+  <si>
+    <t xml:space="preserve">广西</t>
+  </si>
+  <si>
+    <t xml:space="preserve">海南</t>
+  </si>
+  <si>
+    <t xml:space="preserve">重庆</t>
+  </si>
+  <si>
+    <t xml:space="preserve">四川</t>
+  </si>
+  <si>
+    <t xml:space="preserve">贵州</t>
+  </si>
+  <si>
+    <t xml:space="preserve">云南</t>
+  </si>
+  <si>
+    <t xml:space="preserve">西藏</t>
+  </si>
+  <si>
+    <t xml:space="preserve">陕西</t>
+  </si>
+  <si>
+    <t xml:space="preserve">甘肃</t>
+  </si>
+  <si>
+    <t xml:space="preserve">青海</t>
+  </si>
+  <si>
+    <t xml:space="preserve">宁夏</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新疆</t>
   </si>
 </sst>
 </file>

</xml_diff>